<commit_message>
docs: README with architecture, scale and cost strategy, write-up, screenshots; smoke test; fixes
- README: setup, pipeline stages, scale strategy, cost optimisation,
  accuracy, measured numbers, dashboard tour, public API, deployment
- scripts/smoke.ts: end-to-end HTTP check usable against the live demo
- products table: correlated subqueries reference the outer table by name
  (variant counts, prices, photos and translations were rendering empty)
- rows table orders issues by severity; storefront pool sets its
  statement timeout via the startup packet; metadataBase set
- samples: ground-truth categories aligned to the taxonomy (generator
  asserts it); screenshots captured with headless Chromium
</commit_message>
<xml_diff>
--- a/samples/messy-120.xlsx
+++ b/samples/messy-120.xlsx
@@ -518,7 +518,7 @@
         <v>Thick memory foam kneeling pad with a wipe clean cover and a carry handle. Saves knees during planting and weeding and doubles as a seat cushion for camping. Dries quickly after rain.</v>
       </c>
       <c r="E5" t="str">
-        <v>Home &amp; Garden &gt; Lawn &amp; Garden &gt; Gardening &gt; Gardening Accessories</v>
+        <v>Home &amp; Garden &gt; Lawn &amp; Garden &gt; Gardening</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -565,7 +565,7 @@
         <v>Slatted soap dish in bamboo that drains freely so bars dry between uses. Sealed with a plant-based oil. Rinse under the tap and air dry.</v>
       </c>
       <c r="E6" t="str">
-        <v>Home &amp; Garden &gt; Bathroom Accessories &gt; Soap Dishes &amp; Holders</v>
+        <v>Home &amp; Garden &gt; Bathroom Accessories &gt; Soap Dishes &amp; Dispensers</v>
       </c>
       <c r="F6" t="str">
         <v>Bathhouse</v>
@@ -753,7 +753,7 @@
         <v>Floating wall shelf in solid pine with a hidden steel bracket and all fixings included. Holds up to 10 kg of books when mounted into masonry or studs. Sanded smooth and left unfinished for painting or oiling.</v>
       </c>
       <c r="E10" t="str">
-        <v>Furniture &gt; Shelving &gt; Wall Shelves &amp; Ledges</v>
+        <v>Furniture &gt; Shelving</v>
       </c>
       <c r="F10" t="str">
         <v>Hinterland</v>
@@ -800,7 +800,7 @@
         <v>Floating wall shelf in solid pine with a hidden steel bracket and all fixings included. Holds up to 10 kg of books when mounted into masonry or studs. Sanded smooth and left unfinished for painting or oiling.</v>
       </c>
       <c r="E11" t="str">
-        <v>Furniture &gt; Shelving &gt; Wall Shelves &amp; Ledges</v>
+        <v>Furniture &gt; Shelving</v>
       </c>
       <c r="F11" t="str">
         <v>Hinterland</v>
@@ -1076,7 +1076,7 @@
         <v>Warm white LED string lights on a dark green cable with an IP44 transformer, rated for covered outdoor areas. 8 lighting modes with a memory function. Plug-in, with a 3 m lead cable.</v>
       </c>
       <c r="E17" t="str">
-        <v>Home &amp; Garden &gt; Lighting &gt; Lighting Fixtures &gt; String Lights</v>
+        <v>Home &amp; Garden &gt; Lighting &gt; String Lights</v>
       </c>
       <c r="F17" t="str">
         <v>Lumo</v>
@@ -1123,7 +1123,7 @@
         <v>Warm white LED string lights on a dark green cable with an IP44 transformer, rated for covered outdoor areas. 8 lighting modes with a memory function. Plug-in, with a 3 m lead cable.</v>
       </c>
       <c r="E18" t="str">
-        <v>Home &amp; Garden &gt; Lighting &gt; Lighting Fixtures &gt; String Lights</v>
+        <v>Home &amp; Garden &gt; Lighting &gt; String Lights</v>
       </c>
       <c r="F18" t="str">
         <v>Lumo</v>
@@ -1405,7 +1405,7 @@
         <v>Herringbone throw in 100% merino wool, woven in Scotland on traditional looms and finished with a fringed edge. Generous 130 x 180 cm size for sofas and beds. Dry clean only.</v>
       </c>
       <c r="E24" t="str">
-        <v>Home &amp; Garden &gt; Linens &amp; Bedding &gt; Blankets</v>
+        <v>Home &amp; Garden &gt; Linens &amp; Bedding &gt; Bedding &gt; Blankets</v>
       </c>
       <c r="F24" t="str">
         <v>Hinterland</v>
@@ -1452,7 +1452,7 @@
         <v>27 cm dinner plate in vitrified stoneware with a raised rim and a matte outer edge. Chip-resistant and dishwasher-safe for daily use. Made to be mixed with the rest of the range.</v>
       </c>
       <c r="E25" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Plates</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Dinnerware &gt; Plates</v>
       </c>
       <c r="F25" t="str">
         <v>Casa Tierra</v>
@@ -1499,7 +1499,7 @@
         <v>27 cm dinner plate in vitrified stoneware with a raised rim and a matte outer edge. Chip-resistant and dishwasher-safe for daily use. Made to be mixed with the rest of the range.</v>
       </c>
       <c r="E26" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Plates</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Dinnerware &gt; Plates</v>
       </c>
       <c r="F26" t="str">
         <v>Casa Tierra</v>
@@ -1546,7 +1546,7 @@
         <v>Set of three cooking spoons carved from olive wood and hand-finished with food-grade oil. The dense grain resists staining and will not scratch non-stick pans. Hand wash and re-oil occasionally.</v>
       </c>
       <c r="E27" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils &gt; Cooking Utensils</v>
       </c>
       <c r="F27" t="str">
         <v>Oliva</v>
@@ -1593,7 +1593,7 @@
         <v>Pre-seasoned cast-iron skillet with two pour spouts and a helper handle. Oven-safe to 260 °C and induction compatible, it goes from hob to oven to table. Builds a natural non-stick surface with use.</v>
       </c>
       <c r="E28" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Cookware &gt; Skillets &amp; Frying Pans</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Cookware &gt; Pots &amp; Pans</v>
       </c>
       <c r="F28" t="str">
         <v>Oliva</v>
@@ -1640,7 +1640,7 @@
         <v>Pre-seasoned cast-iron skillet with two pour spouts and a helper handle. Oven-safe to 260 °C and induction compatible, it goes from hob to oven to table. Builds a natural non-stick surface with use.</v>
       </c>
       <c r="E29" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Cookware &gt; Skillets &amp; Frying Pans</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Cookware &gt; Pots &amp; Pans</v>
       </c>
       <c r="F29" t="str">
         <v>Oliva</v>
@@ -1687,7 +1687,7 @@
         <v>Set of three spatulas in BPA-free silicone over a stainless steel core. Heat-resistant to 230 °C and safe on non-stick coatings. Dishwasher-safe and one-piece, so nothing collects in the seams.</v>
       </c>
       <c r="E30" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils &gt; Cooking Utensils</v>
       </c>
       <c r="F30" t="str">
         <v>Oliva</v>
@@ -1734,7 +1734,7 @@
         <v>Set of three spatulas in BPA-free silicone over a stainless steel core. Heat-resistant to 230 °C and safe on non-stick coatings. Dishwasher-safe and one-piece, so nothing collects in the seams.</v>
       </c>
       <c r="E31" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils &gt; Cooking Utensils</v>
       </c>
       <c r="F31" t="str">
         <v>Oliva</v>
@@ -1781,7 +1781,7 @@
         <v>Set of three spatulas in BPA-free silicone over a stainless steel core. Heat-resistant to 230 °C and safe on non-stick coatings. Dishwasher-safe and one-piece, so nothing collects in the seams.</v>
       </c>
       <c r="E32" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils &gt; Cooking Utensils</v>
       </c>
       <c r="F32" t="str">
         <v>Oliva</v>
@@ -1828,7 +1828,7 @@
         <v>Tipper truck in beech wood with rubber wheels that are quiet on wooden floors and a tipping bed that locks upright. Finished with clear water-based lacquer. Small parts: suitable from 3 years.</v>
       </c>
       <c r="E33" t="str">
-        <v>Toys &amp; Games &gt; Toys &gt; Toy Vehicles</v>
+        <v>Toys &amp; Games &gt; Toys &gt; Wooden Toys</v>
       </c>
       <c r="F33" t="str">
         <v>Little Larch</v>
@@ -2063,7 +2063,7 @@
         <v>Table runner in 100% organic cotton with a woven stripe and hand-knotted tassels at both ends. Measures 40 x 150 cm and is machine washable at 40 °C. The natural dyes mellow gently over time.</v>
       </c>
       <c r="E38" t="str">
-        <v>Home &amp; Garden &gt; Linens &amp; Bedding &gt; Table Linens &gt; Table Runners</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Table Linens</v>
       </c>
       <c r="F38" t="str">
         <v>Hinterland</v>
@@ -2205,7 +2205,7 @@
 Machine washable at 30 °C and dries on the line. Suitable for medium and large dogs.</v>
       </c>
       <c r="E41" t="str">
-        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Dog Supplies &gt; Dog Toys</v>
+        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Pet Toys</v>
       </c>
       <c r="F41" t="str">
         <v>Pawfolk</v>
@@ -2252,7 +2252,7 @@
         <v>Writing pad of 80 sheets in 100% recycled paper, ruled with a faint grey line and glued at the head for clean tearing. Backed with a thick grey board. Available in A4 and A5.</v>
       </c>
       <c r="E42" t="str">
-        <v>Office Supplies &gt; General Office Supplies &gt; Paper Products &gt; Notepads</v>
+        <v>Office Supplies &gt; General Office Supplies &gt; Paper &gt; Notebooks &amp; Notepads</v>
       </c>
       <c r="F42" t="str">
         <v>Folio</v>
@@ -2299,7 +2299,7 @@
         <v>Writing pad of 80 sheets in 100% recycled paper, ruled with a faint grey line and glued at the head for clean tearing. Backed with a thick grey board. Available in A4 and A5.</v>
       </c>
       <c r="E43" t="str">
-        <v>Office Supplies &gt; General Office Supplies &gt; Paper Products &gt; Notepads</v>
+        <v>Office Supplies &gt; General Office Supplies &gt; Paper &gt; Notebooks &amp; Notepads</v>
       </c>
       <c r="F43" t="str">
         <v>Folio</v>
@@ -2346,7 +2346,7 @@
         <v>Fountain pen with a medium steel nib and a brushed aluminium barrel, converter included for bottled ink. Takes standard international cartridges as well. Writes wet with a slight line variation.</v>
       </c>
       <c r="E44" t="str">
-        <v>Office Supplies &gt; General Office Supplies &gt; Writing &amp; Drawing Instruments &gt; Pens</v>
+        <v>Office Supplies &gt; Writing Instruments &gt; Pens</v>
       </c>
       <c r="F44" t="str">
         <v>Folio</v>
@@ -2393,7 +2393,7 @@
         <v>900 ml teapot in glazed stoneware with a removable stainless steel infuser and a drip-free spout. The lid locks into the handle so it stays put while pouring. Hand wash only.</v>
       </c>
       <c r="E45" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Coffee &amp; Tea Sets</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Serveware &gt; Teapots</v>
       </c>
       <c r="F45" t="str">
         <v/>
@@ -2440,7 +2440,7 @@
         <v>Plant stand in powder-coated steel with a round top that takes pots up to 25 cm across. Suitable for indoor use; the slim legs keep it light enough to move with the plant on it. Comes in two heights.</v>
       </c>
       <c r="E46" t="str">
-        <v>Home &amp; Garden &gt; Decor &gt; Plant Stands</v>
+        <v>Home &amp; Garden &gt; Decor</v>
       </c>
       <c r="F46" t="str">
         <v>Form &amp; Fibre</v>
@@ -2957,7 +2957,7 @@
         <v>Desk organiser in oak veneer with five compartments for pens, phone, cards and clips, felt lined to stop things rattling. Sits flat on the desk without feet. Dust with a dry cloth.</v>
       </c>
       <c r="E57" t="str">
-        <v>Office Supplies &gt; General Office Supplies &gt; Desk Organizers</v>
+        <v>Office Supplies &gt; Desk Accessories</v>
       </c>
       <c r="F57" t="str">
         <v>N/A</v>
@@ -3333,7 +3333,7 @@
         <v>Soft plush rabbit, 30 cm tall, with embroidered eyes rather than buttons and long floppy ears. Machine washable at 30 °C in a wash bag. Filled with recycled fibre.</v>
       </c>
       <c r="E65" t="str">
-        <v>Toys &amp; Games &gt; Toys &gt; Stuffed Animals</v>
+        <v>Toys &amp; Games &gt; Toys &gt; Dolls &amp; Stuffed Animals</v>
       </c>
       <c r="F65" t="str">
         <v>Little Larch</v>
@@ -3380,7 +3380,7 @@
         <v>Soft plush rabbit, 30 cm tall, with embroidered eyes rather than buttons and long floppy ears. Machine washable at 30 °C in a wash bag. Filled with recycled fibre.</v>
       </c>
       <c r="E66" t="str">
-        <v>Toys &amp; Games &gt; Toys &gt; Stuffed Animals</v>
+        <v>Toys &amp; Games &gt; Toys &gt; Dolls &amp; Stuffed Animals</v>
       </c>
       <c r="F66" t="str">
         <v>Little Larch</v>
@@ -3521,7 +3521,7 @@
         <v>Heavy stoneware pet bowl with a non-slip base and a wide rim that keeps whiskers clear. Dishwasher-safe and glazed with a lead-free finish. Three sizes from cat to large dog.</v>
       </c>
       <c r="E69" t="str">
-        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Pet Bowls, Feeders &amp; Waterers</v>
+        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Pet Bowls &amp; Feeders</v>
       </c>
       <c r="F69" t="str">
         <v>Pawfolk</v>
@@ -3756,7 +3756,7 @@
         <v>Set of 24 stacking blocks in beech wood, coloured with water-based paint and sanded with rounded edges. Suitable from 12 months. Comes in a cotton drawstring bag.</v>
       </c>
       <c r="E74" t="str">
-        <v>Toys &amp; Games &gt; Toys &gt; Building Toys &gt; Stacking Blocks</v>
+        <v>Toys &amp; Games &gt; Toys &gt; Building Toys</v>
       </c>
       <c r="F74" t="str">
         <v>Little Larch</v>
@@ -3988,7 +3988,7 @@
         <v>Hand trowel with a stainless steel blade and an ash handle that is oiled rather than varnished for better grip. The blade has depth marks for bulbs and a sharpened edge for cutting roots. Leather loop for hanging.</v>
       </c>
       <c r="E76" t="str">
-        <v>Home &amp; Garden &gt; Lawn &amp; Garden &gt; Gardening &gt; Gardening Tools</v>
+        <v>Home &amp; Garden &gt; Lawn &amp; Garden &gt; Gardening &gt; Gardening Tools &gt; Hand Trowels</v>
       </c>
       <c r="F76" t="str">
         <v>Greenhand</v>
@@ -4223,7 +4223,7 @@
         <v>Chunky 12 pieces farm puzzle cut from birch plywood with a printed guide underneath each piece. The knobs are sized for small hands. Wipe clean with a damp cloth.</v>
       </c>
       <c r="E81" t="str">
-        <v>Toys &amp; Games &gt; Puzzles &gt; Jigsaw Puzzles</v>
+        <v>Toys &amp; Games &gt; Games &gt; Puzzles</v>
       </c>
       <c r="F81" t="str">
         <v>Little Larch</v>
@@ -4602,7 +4602,7 @@
         <v>&lt;p&gt;&lt;b&gt;Single-hole pencil sharpener machined from solid brass with a replacement blade included in the box.&lt;p&gt;The weight keeps it steady on the desk. Fits standard and jumbo pencils.&lt;br&gt;&lt;i&gt;See notes</v>
       </c>
       <c r="E89" t="str">
-        <v>Office Supplies &gt; General Office Supplies &gt; Writing &amp; Drawing Instruments &gt; Pencil Sharpeners</v>
+        <v>Office Supplies &gt; Writing Instruments</v>
       </c>
       <c r="F89" t="str">
         <v/>
@@ -4649,7 +4649,7 @@
         <v>Deep stoneware serving bowl with a food-safe glaze in speckled oatmeal and a hand-painted metallic rim. Dishwasher-safe on a normal cycle. Sized for salads, pasta and family-style sides.</v>
       </c>
       <c r="E90" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Serveware</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Serveware &gt; Serving Bowls</v>
       </c>
       <c r="F90" t="str">
         <v>Casa Tierra</v>
@@ -4696,7 +4696,7 @@
         <v>Two-tier shower caddy in rust-resistant coated steel that hangs over the shower head with no drilling. Each shelf holds three bottles and has hooks for razors and loofahs. Adjustable hanger for different pipe angles.</v>
       </c>
       <c r="E91" t="str">
-        <v>Home &amp; Garden &gt; Bathroom Accessories &gt; Shower Caddies</v>
+        <v>Home &amp; Garden &gt; Bathroom Accessories</v>
       </c>
       <c r="F91" t="str">
         <v>Bathhouse</v>
@@ -5025,7 +5025,7 @@
         <v>Heavy stoneware pet bowl with a non-slip base and a wide rim that keeps whiskers clear. Dishwasher-safe and glazed with a lead-free finish. Three sizes from cat to large dog.</v>
       </c>
       <c r="E98" t="str">
-        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Pet Bowls, Feeders &amp; Waterers</v>
+        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Pet Bowls &amp; Feeders</v>
       </c>
       <c r="F98" t="str">
         <v>Pawfolk</v>
@@ -5072,7 +5072,7 @@
         <v>150 cm dog leash in woven polyester webbing with reflective stitching along both edges and a padded handle. The trigger clip is solid brass. Wipe clean.</v>
       </c>
       <c r="E99" t="str">
-        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Dog Supplies &gt; Dog Leashes</v>
+        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Dog Supplies</v>
       </c>
       <c r="F99" t="str">
         <v>Pawfolk</v>
@@ -5119,7 +5119,7 @@
         <v>150 cm dog leash in woven polyester webbing with reflective stitching along both edges and a padded handle. The trigger clip is solid brass. Wipe clean.</v>
       </c>
       <c r="E100" t="str">
-        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Dog Supplies &gt; Dog Leashes</v>
+        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Dog Supplies</v>
       </c>
       <c r="F100" t="str">
         <v>Pawfolk</v>
@@ -5166,7 +5166,7 @@
         <v>150 cm dog leash in woven polyester webbing with reflective stitching along both edges and a padded handle. The trigger clip is solid brass. Wipe clean.</v>
       </c>
       <c r="E101" t="str">
-        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Dog Supplies &gt; Dog Leashes</v>
+        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Dog Supplies</v>
       </c>
       <c r="F101" t="str">
         <v>Pawfolk</v>
@@ -5213,7 +5213,7 @@
         <v>Plant stand in powder-coated steel with a round top that takes pots up to 25 cm across. Suitable for indoor use; the slim legs keep it light enough to move with the plant on it. Comes in two heights.</v>
       </c>
       <c r="E102" t="str">
-        <v>Home &amp; Garden &gt; Decor &gt; Plant Stands</v>
+        <v>Home &amp; Garden &gt; Decor</v>
       </c>
       <c r="F102" t="str">
         <v>Form &amp; Fibre</v>
@@ -5260,7 +5260,7 @@
         <v>Balloon whisk in 18/8 stainless steel with twelve wires and a sealed, weighted handle. Dishwasher-safe and rust-resistant. 30 cm long, so it reaches the corners of a tall jug.</v>
       </c>
       <c r="E103" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Kitchen Tools &amp; Utensils &gt; Cooking Utensils</v>
       </c>
       <c r="F103" t="str">
         <v>Oliva</v>
@@ -5542,7 +5542,7 @@
         <v>Single line diamond kite in ripstop nylon with a 2 m tail and fibreglass spars. Flies in light wind and packs into a sleeve. 30 m line on a winder included.</v>
       </c>
       <c r="E109" t="str">
-        <v>Toys &amp; Games &gt; Outdoor Play Equipment &gt; Kites</v>
+        <v>Toys &amp; Games &gt; Toys &gt; Outdoor Toys</v>
       </c>
       <c r="F109" t="str">
         <v>Little Larch</v>
@@ -5589,7 +5589,7 @@
         <v>Single line diamond kite in ripstop nylon with a 2 m tail and fibreglass spars. Flies in light wind and packs into a sleeve. 30 m line on a winder included.</v>
       </c>
       <c r="E110" t="str">
-        <v>Toys &amp; Games &gt; Outdoor Play Equipment &gt; Kites</v>
+        <v>Toys &amp; Games &gt; Toys &gt; Outdoor Toys</v>
       </c>
       <c r="F110" t="str">
         <v>Little Larch</v>
@@ -5636,7 +5636,7 @@
         <v>60 cm scratching post wrapped in natural sisal on a solid base of carpeted MDF. Heavy enough that it will not tip when a large cat leans into it. Replacement sisal sleeves are available.</v>
       </c>
       <c r="E111" t="str">
-        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Cat Supplies &gt; Cat Furniture</v>
+        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Cat Supplies</v>
       </c>
       <c r="F111" t="str">
         <v>Pawfolk</v>
@@ -5683,7 +5683,7 @@
         <v>Bedside table with one drawer and an open shelf, in ash veneer over an engineered board with solid ash legs. The drawer runs on wooden runners and has a cut-out pull instead of a handle. Arrives assembled.</v>
       </c>
       <c r="E112" t="str">
-        <v>Furniture &gt; Tables &gt; Nightstands</v>
+        <v>Furniture &gt; Tables &gt; Side Tables</v>
       </c>
       <c r="F112" t="str">
         <v>Hinterland</v>
@@ -5730,7 +5730,7 @@
         <v>Round side table in solid oak with a turned pedestal base and a hand-oiled top. The timber is FSC-certified and finished without stain, so the grain shows through. Delivered flat-packed with two fixings.</v>
       </c>
       <c r="E113" t="str">
-        <v>Furniture &gt; Tables &gt; Accent Tables &gt; End Tables</v>
+        <v>Furniture &gt; Tables &gt; Side Tables</v>
       </c>
       <c r="F113" t="str">
         <v>Hinterland</v>
@@ -5777,7 +5777,7 @@
         <v>Heavy stoneware pet bowl with a non-slip base and a wide rim that keeps whiskers clear. Dishwasher-safe and glazed with a lead-free finish. Three sizes from cat to large dog.</v>
       </c>
       <c r="E114" t="str">
-        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Pet Bowls, Feeders &amp; Waterers</v>
+        <v>Animals &amp; Pet Supplies &gt; Pet Supplies &gt; Pet Bowls &amp; Feeders</v>
       </c>
       <c r="F114" t="str">
         <v>Pawfolk</v>
@@ -5824,7 +5824,7 @@
         <v>Round side table in solid oak with a turned pedestal base and a hand-oiled top. The timber is FSC-certified and finished without stain, so the grain shows through. Delivered flat-packed with two fixings.</v>
       </c>
       <c r="E115" t="str">
-        <v>Furniture &gt; Tables &gt; Accent Tables &gt; End Tables</v>
+        <v>Furniture &gt; Tables &gt; Side Tables</v>
       </c>
       <c r="F115" t="str">
         <v>Hinterland</v>
@@ -5871,7 +5871,7 @@
         <v>Two-tier shower caddy in rust-resistant coated steel that hangs over the shower head with no drilling. Each shelf holds three bottles and has hooks for razors and loofahs. Adjustable hanger for different pipe angles.</v>
       </c>
       <c r="E116" t="str">
-        <v>Home &amp; Garden &gt; Bathroom Accessories &gt; Shower Caddies</v>
+        <v>Home &amp; Garden &gt; Bathroom Accessories</v>
       </c>
       <c r="F116" t="str">
         <v>Bathhouse</v>
@@ -6153,7 +6153,7 @@
         <v>Deep stoneware serving bowl with a food-safe glaze in speckled oatmeal and a hand-painted metallic rim. Dishwasher-safe on a normal cycle. Sized for salads, pasta and family-style sides.</v>
       </c>
       <c r="E122" t="str">
-        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Serveware</v>
+        <v>Home &amp; Garden &gt; Kitchen &amp; Dining &gt; Tableware &gt; Serveware &gt; Serving Bowls</v>
       </c>
       <c r="F122" t="str">
         <v>Casa Tierra</v>
@@ -6200,7 +6200,7 @@
         <v>Round side table in solid oak with a turned pedestal base and a hand-oiled top. The timber is FSC-certified and finished without stain, so the grain shows through. Delivered flat-packed with two fixings.</v>
       </c>
       <c r="E123" t="str">
-        <v>Furniture &gt; Tables &gt; Accent Tables &gt; End Tables</v>
+        <v>Furniture &gt; Tables &gt; Side Tables</v>
       </c>
       <c r="F123" t="str">
         <v>Hinterland</v>

</xml_diff>